<commit_message>
added workers to spreadsheet
</commit_message>
<xml_diff>
--- a/UploadTemplate.xlsx
+++ b/UploadTemplate.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/hammertech-worker-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F507D574-B171-48CF-BDD1-4E8709BC09C6}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="2580" windowWidth="21600" windowHeight="11175" activeTab="2" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
     <sheet name="Projects" sheetId="2" r:id="rId2"/>
     <sheet name="EmployerProfiles" sheetId="3" r:id="rId3"/>
+    <sheet name="Workers" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
   <si>
     <t>Email Address</t>
   </si>
@@ -95,6 +96,33 @@
   </si>
   <si>
     <t>Postal Code</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Job Title ID</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>Suburb</t>
+  </si>
+  <si>
+    <t>Postcode</t>
+  </si>
+  <si>
+    <t>Internal Id</t>
+  </si>
+  <si>
+    <t>Project ID</t>
+  </si>
+  <si>
+    <t>Employer ID</t>
   </si>
 </sst>
 </file>
@@ -130,10 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -473,22 +498,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -503,25 +528,25 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -536,32 +561,88 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63FD6A01-0607-4804-B827-1FFE6B736FC7}">
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="13" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ability to add user to all projects at once
</commit_message>
<xml_diff>
--- a/UploadTemplate.xlsx
+++ b/UploadTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/hammertech-worker-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F507D574-B171-48CF-BDD1-4E8709BC09C6}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{810D9C35-8E68-4B86-A476-DF9256162583}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -496,6 +496,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9163D3E5-3974-4D02-94C9-F4EF4023A67A}">
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
added user functionality for specific permissions needed with all functionality
</commit_message>
<xml_diff>
--- a/UploadTemplate.xlsx
+++ b/UploadTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/hammertech-worker-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{810D9C35-8E68-4B86-A476-DF9256162583}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0BFBF8A-CFA2-4107-9A97-AA29617CDD66}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
   <si>
     <t>Email Address</t>
   </si>
@@ -123,6 +123,21 @@
   </si>
   <si>
     <t>Employer ID</t>
+  </si>
+  <si>
+    <t>Project Admin</t>
+  </si>
+  <si>
+    <t>Individual Daily Report</t>
+  </si>
+  <si>
+    <t>Daily Report Admin</t>
+  </si>
+  <si>
+    <t>Site Notifications</t>
+  </si>
+  <si>
+    <t>Confidential Data</t>
   </si>
 </sst>
 </file>
@@ -494,16 +509,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9163D3E5-3974-4D02-94C9-F4EF4023A67A}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,6 +542,21 @@
       </c>
       <c r="F1" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added column to excel
</commit_message>
<xml_diff>
--- a/UploadTemplate.xlsx
+++ b/UploadTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/hammertech-worker-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0BFBF8A-CFA2-4107-9A97-AA29617CDD66}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AF7BFCE-BDDE-494E-8A38-9482A00DE8C2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>Email Address</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>Confidential Data</t>
+  </si>
+  <si>
+    <t>Mobile</t>
   </si>
 </sst>
 </file>
@@ -635,7 +638,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63FD6A01-0607-4804-B827-1FFE6B736FC7}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
@@ -643,7 +646,7 @@
     <col min="7" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -682,6 +685,9 @@
       </c>
       <c r="M1" t="s">
         <v>27</v>
+      </c>
+      <c r="N1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>